<commit_message>
(Component selection and documentation) bomV2 and hardware overview
</commit_message>
<xml_diff>
--- a/BOM/Vital-Link-BOM2-V1.xlsx
+++ b/BOM/Vital-Link-BOM2-V1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GITHUB_desktop\Vital-link-hardware\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GitHub\Vital-link-hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9232E352-D508-4709-8564-2D26FD8B2C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E87B4E-BA45-445E-B536-E863CC0967F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>BOM #:</t>
   </si>
@@ -107,22 +107,70 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>https://www.digikey.ca/en/mylists/list/YB1AS4802V</t>
-  </si>
-  <si>
-    <t>HERE'S A LIST OF ALL THE COMPONENTS on digikey</t>
-  </si>
-  <si>
-    <t>https://www.mouser.com/ProductDetail/Analog-Devices-Maxim-Integrated/MAX30003WING?qs=55YtniHzbhB8FzqvuARmyw%3D%3D&amp;mgh=1&amp;utm_id=22260989504&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_marketing_tactic=amercorp&amp;gad_source=1&amp;gad_campaignid=22264895254&amp;gbraid=0AAAAADn_wf3ueVpY8hDHNSFXSMw5zAMcE&amp;gclid=Cj0KCQiA1JLLBhCDARIsAAVfy7j557U5wdZEqoSzD3K6uXroa0ZPy_YSwdKYwT6Wu6fiLRe04yLQQgsaAoOyEALw_wcB</t>
-  </si>
-  <si>
-    <t>MAX30003WING</t>
+    <t>ECG specific board</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005009180943063.html?spm=a2g0o.productlist.main.9.21915c61oF6QAf&amp;algo_pvid=5f32d17c-5085-463e-bf55-f579c014c13a&amp;algo_exp_id=5f32d17c-5085-463e-bf55-f579c014c13a-8&amp;pdp_ext_f=%7B%22order%22%3A%22132%22%2C%22spu_best_type%22%3A%22order%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis!CAD!9.78!4.79!!!47.86!23.45!%402103129017688064390718772ebb33!12000048217403188!sea!CA!3114729883!ACX!1!0!n_tag%3A-29919%3Bd%3A5279d241%3Bm03_new_user%3A-29894&amp;curPageLogUid=4L9aGEGiNkMr&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005009180943063%7C_p_origin_prod%3A#nav-review</t>
+  </si>
+  <si>
+    <t>80mAh Lithium battery</t>
+  </si>
+  <si>
+    <t>1Piece 3.7V 80mAh 501220 Rechargeable Lithium Battery For Headsets 3D Glasses Sports Bracelets More Gadgets</t>
+  </si>
+  <si>
+    <t>8% off on 10 items.
+80mAH Battery, expected delivery time is 1 month</t>
+  </si>
+  <si>
+    <t>https://www.mouser.ca/ProductDetail/Analog-Devices-Maxim-Integrated/MAX30003WING?qs=55YtniHzbhB8FzqvuARmyw%3D%3D</t>
+  </si>
+  <si>
+    <t>MAX30003WING#</t>
   </si>
   <si>
     <t>Data Conversion IC Development Tools ECG AFE feather board</t>
   </si>
   <si>
-    <t>ECG specific board</t>
+    <t>https://www.mouser.ca/ProductDetail/SparkFun/SEN-12969?qs=WyAARYrbSnaajKSHkjOGnw%3D%3D&amp;srsltid=AfmBOopLlhnPtYg_Z8E7CQDvXOVRvZXciZKFLqnQvesH_fLeNzKnnWjU</t>
+  </si>
+  <si>
+    <t>SEN-12969</t>
+  </si>
+  <si>
+    <t>Biometric Sensors Disposable Surface EMG/ECG/EKG Electrode - 24mm (10 pack)</t>
+  </si>
+  <si>
+    <t>https://www.alibaba.com/product-detail/3-Feet-Standard-4-0mm-Female_1600464585377.html?spm=a2700.details.you_may_like.2.38db2c99CN4RWw</t>
+  </si>
+  <si>
+    <t>QB-24031121</t>
+  </si>
+  <si>
+    <t>3 feet 4.0mm female ECG snap buttons</t>
+  </si>
+  <si>
+    <t>https://www.alibaba.com/product-detail/3-Claw-4-0-Medical-Electrode_1601678125336.html?spm=a2700.prosearch.normal_offer.d_title.5b2d67afx0eMoD&amp;priceId=5565a05ffcc44744bc23fdbad2025240</t>
+  </si>
+  <si>
+    <t>3-Claw 4.0 Medical Electrode Snap Easy-to-solder PCB ECG</t>
+  </si>
+  <si>
+    <t>S-26011001</t>
+  </si>
+  <si>
+    <t>The main focus on this BOM is to order components with extended shipping time ( from china)</t>
+  </si>
+  <si>
+    <t>Make sure to press get sample
+to allow us to order 10</t>
+  </si>
+  <si>
+    <t>Backup for above with another distributor. 
+As well as has longer shipping time</t>
+  </si>
+  <si>
+    <t>3 x 10pack for 0$ shipping</t>
   </si>
 </sst>
 </file>
@@ -132,7 +180,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -181,51 +229,77 @@
       <name val="Roboto"/>
     </font>
     <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF333333"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -244,8 +318,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -345,13 +425,9 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
+      <left/>
       <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -362,30 +438,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
@@ -393,10 +445,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -404,93 +457,83 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -504,6 +547,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>314921</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>552523</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8BD20C1D-C76E-4DCB-96D2-7527FB746473}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20793075" y="2590800"/>
+          <a:ext cx="4267796" cy="523948"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -707,13 +799,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.42578125" customWidth="1"/>
     <col min="2" max="2" width="79.140625" customWidth="1"/>
     <col min="3" max="3" width="34.5703125" customWidth="1"/>
-    <col min="4" max="4" width="28.28515625" customWidth="1"/>
+    <col min="4" max="4" width="96.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="31.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -722,37 +814,35 @@
         <v>0</v>
       </c>
       <c r="B1" s="1">
-        <v>1</v>
-      </c>
-      <c r="C1" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="D1" s="17"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="C1" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
-    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="26" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -767,7 +857,7 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="39"/>
+      <c r="A4" s="27"/>
       <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
@@ -779,7 +869,7 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="39"/>
+      <c r="A5" s="27"/>
       <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
@@ -791,7 +881,7 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="40"/>
+      <c r="A6" s="28"/>
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
@@ -845,239 +935,327 @@
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="10" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28">
+      <c r="A11" s="12">
         <v>1</v>
       </c>
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="15">
+        <v>1</v>
+      </c>
+      <c r="F11" s="16">
+        <v>0</v>
+      </c>
+      <c r="G11" s="17">
+        <v>64.81</v>
+      </c>
+      <c r="H11" s="16">
+        <f>(G11*E11)</f>
+        <v>64.81</v>
+      </c>
+      <c r="I11" s="18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="12">
+        <v>2</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="15">
+        <v>3</v>
+      </c>
+      <c r="F12" s="16">
+        <v>0</v>
+      </c>
+      <c r="G12" s="16">
+        <v>14.83</v>
+      </c>
+      <c r="H12" s="16">
+        <f>(G12*E12)</f>
+        <v>44.49</v>
+      </c>
+      <c r="I12" s="20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="21">
+        <v>3</v>
+      </c>
+      <c r="B13" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="22">
+        <v>10</v>
+      </c>
+      <c r="F13" s="22">
+        <v>0</v>
+      </c>
+      <c r="G13" s="22">
+        <v>1.39</v>
+      </c>
+      <c r="H13" s="16">
+        <f>(G13*E13)</f>
+        <v>13.899999999999999</v>
+      </c>
+      <c r="I13" s="41" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="39" x14ac:dyDescent="0.25">
+      <c r="A14" s="38">
+        <v>4</v>
+      </c>
+      <c r="B14" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="22">
+        <v>10</v>
+      </c>
+      <c r="F14" s="22">
+        <v>0</v>
+      </c>
+      <c r="G14" s="22">
+        <v>0.30409999999999998</v>
+      </c>
+      <c r="H14" s="16">
+        <f>(G14*E14)</f>
+        <v>3.0409999999999999</v>
+      </c>
+      <c r="I14" s="39" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="39" x14ac:dyDescent="0.25">
+      <c r="A15" s="12">
+        <v>4</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="45" t="s">
+      <c r="D15" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="46" t="s">
+      <c r="E15" s="15">
+        <v>10</v>
+      </c>
+      <c r="F15" s="16">
+        <v>5.34</v>
+      </c>
+      <c r="G15" s="16">
+        <v>4.79</v>
+      </c>
+      <c r="H15" s="16">
+        <f>(G15*E15)*0.92+F15</f>
+        <v>49.408000000000001</v>
+      </c>
+      <c r="I15" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="47" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28">
-        <v>3</v>
-      </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="12"/>
-    </row>
-    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="28">
-        <v>4</v>
-      </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="12"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="18">
-        <v>5</v>
-      </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="19"/>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="28">
-        <v>6</v>
-      </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="12"/>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="28">
-        <v>7</v>
-      </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="12"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="23"/>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="28"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="12"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="23"/>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="28"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="12"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="23"/>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="12"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="23"/>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="12"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="23"/>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="12"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="29">
+        <f>SUM(H11:H20)</f>
+        <v>175.649</v>
+      </c>
+      <c r="G21" s="30"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="4"/>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
-      <c r="C22" s="14"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="5"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="F22" s="41">
-        <f>SUM(H11:H21)</f>
-        <v>0</v>
-      </c>
-      <c r="G22" s="42"/>
-      <c r="H22" s="43"/>
+      <c r="E22" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" s="32">
+        <f>F21*0.12</f>
+        <v>21.07788</v>
+      </c>
+      <c r="G22" s="33"/>
+      <c r="H22" s="34"/>
       <c r="I22" s="4"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
-      <c r="C23" s="14"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="5"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="F23" s="41">
-        <f>F22*0.12</f>
-        <v>0</v>
-      </c>
-      <c r="G23" s="42"/>
-      <c r="H23" s="43"/>
+      <c r="E23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" s="35">
+        <f>SUM(F21:H22)</f>
+        <v>196.72687999999999</v>
+      </c>
+      <c r="G23" s="33"/>
+      <c r="H23" s="34"/>
       <c r="I23" s="4"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="14"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="5"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F24" s="44">
-        <f>SUM(F22:H23)</f>
-        <v>0</v>
-      </c>
-      <c r="G24" s="42"/>
-      <c r="H24" s="43"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
+    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="25"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="25"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="25"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="25"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A3:A6"/>
+    <mergeCell ref="F21:H21"/>
     <mergeCell ref="F22:H22"/>
     <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="C1:G2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B13" r:id="rId1" xr:uid="{98C796B6-F63D-4346-9A15-BA0EC73DC79F}"/>
+    <hyperlink ref="B14" r:id="rId2" xr:uid="{74A51A80-5BC3-4785-BCB5-F8B6A6761DA5}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>